<commit_message>
made changes to financial model
</commit_message>
<xml_diff>
--- a/Financial Statement Model Online Walk Through.xlsx
+++ b/Financial Statement Model Online Walk Through.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eipny-my.sharepoint.com/personal/isiaka_energyimpactpartners_com/Documents/Training/Financial Modelling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="491" documentId="13_ncr:1_{DD486496-2B70-447A-98D9-F2E49C8F2BC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47DEB86C-30B6-45FF-95A3-E420938A7885}"/>
+  <xr:revisionPtr revIDLastSave="603" documentId="13_ncr:1_{DD486496-2B70-447A-98D9-F2E49C8F2BC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0CFE351-5DE7-4165-8C60-4C5D3FA154DB}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="11370" tabRatio="736" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="736" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FSM Data Input_Empty" sheetId="66" r:id="rId1"/>
@@ -83,7 +83,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="12">'Rev Build Complete'!$C$2:$R$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="11">'Rev Build Fill '!$C$2:$Q$41</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcCompleted="0"/>
+  <calcPr calcId="191029" calcMode="autoNoTable"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -2499,7 +2499,7 @@
             <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-Increse common stock by stock bsed compenstation
+common stock increases because ever year we get + are prev yr
 </t>
         </r>
       </text>
@@ -3401,7 +3401,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3415" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3419" uniqueCount="335">
   <si>
     <t>Tax rate</t>
   </si>
@@ -4458,6 +4458,15 @@
   <si>
     <t>Repurchases of common stock</t>
   </si>
+  <si>
+    <t>outflow</t>
+  </si>
+  <si>
+    <t>Inflow</t>
+  </si>
+  <si>
+    <t>Rev</t>
+  </si>
 </sst>
 </file>
 
@@ -5168,7 +5177,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="44">
+  <fills count="46">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5398,6 +5407,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD2F2FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -6316,7 +6337,7 @@
     <xf numFmtId="0" fontId="82" fillId="0" borderId="0" applyAlignment="0"/>
     <xf numFmtId="233" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellStyleXfs>
-  <cellXfs count="302">
+  <cellXfs count="305">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="62" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -6749,6 +6770,9 @@
     <xf numFmtId="10" fontId="2" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="63" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="60" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="42" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="44" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="37" fontId="2" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="209">
     <cellStyle name="$" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -53525,11 +53549,26 @@
       <c r="F30" s="3">
         <v>10903</v>
       </c>
-      <c r="G30" s="96"/>
-      <c r="H30" s="96"/>
-      <c r="I30" s="96"/>
-      <c r="J30" s="96"/>
-      <c r="K30" s="96"/>
+      <c r="G30" s="304">
+        <f>G106</f>
+        <v>10722.489599999999</v>
+      </c>
+      <c r="H30" s="304">
+        <f t="shared" ref="H30:K30" si="10">H106</f>
+        <v>11636.785152</v>
+      </c>
+      <c r="I30" s="304">
+        <f t="shared" si="10"/>
+        <v>12729.364789632</v>
+      </c>
+      <c r="J30" s="304">
+        <f t="shared" si="10"/>
+        <v>13917.317683148543</v>
+      </c>
+      <c r="K30" s="304">
+        <f t="shared" si="10"/>
+        <v>15208.603570206933</v>
+      </c>
       <c r="M30" t="s">
         <v>158</v>
       </c>
@@ -53552,23 +53591,23 @@
       </c>
       <c r="G31" s="300">
         <f>G22+G30</f>
-        <v>61703.030399999989</v>
+        <v>72425.51999999999</v>
       </c>
       <c r="H31" s="300">
-        <f t="shared" ref="H31:K31" si="10">H22+H30</f>
-        <v>67297.098528000002</v>
+        <f t="shared" ref="H31:K31" si="11">H22+H30</f>
+        <v>78933.883679999999</v>
       </c>
       <c r="I31" s="300">
-        <f t="shared" si="10"/>
-        <v>72229.51639199999</v>
+        <f t="shared" si="11"/>
+        <v>84958.881181631994</v>
       </c>
       <c r="J31" s="300">
-        <f t="shared" si="10"/>
-        <v>77213.353023047996</v>
+        <f t="shared" si="11"/>
+        <v>91130.670706196543</v>
       </c>
       <c r="K31" s="300">
-        <f t="shared" si="10"/>
-        <v>82541.074381638289</v>
+        <f t="shared" si="11"/>
+        <v>97749.677951845224</v>
       </c>
       <c r="M31" s="16" t="s">
         <v>97</v>
@@ -53592,19 +53631,19 @@
         <v>5126.3999999999996</v>
       </c>
       <c r="H32" s="59">
-        <f t="shared" ref="H32:K32" si="11">G32 *(1+H36)</f>
+        <f t="shared" ref="H32:K32" si="12">G32 *(1+H36)</f>
         <v>5433.9839999999995</v>
       </c>
       <c r="I32" s="59">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>5808.9288959999994</v>
       </c>
       <c r="J32" s="59">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>6209.7449898239993</v>
       </c>
       <c r="K32" s="59">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>6638.2173941218552</v>
       </c>
       <c r="M32" t="s">
@@ -53629,23 +53668,23 @@
       </c>
       <c r="G33" s="300">
         <f>G31+G32</f>
-        <v>66829.430399999983</v>
+        <v>77551.919999999984</v>
       </c>
       <c r="H33" s="300">
-        <f t="shared" ref="H33:K33" si="12">H31+H32</f>
-        <v>72731.082527999999</v>
+        <f t="shared" ref="H33:K33" si="13">H31+H32</f>
+        <v>84367.867679999996</v>
       </c>
       <c r="I33" s="300">
-        <f t="shared" si="12"/>
-        <v>78038.445287999988</v>
+        <f t="shared" si="13"/>
+        <v>90767.810077631992</v>
       </c>
       <c r="J33" s="300">
-        <f t="shared" si="12"/>
-        <v>83423.098012871997</v>
+        <f t="shared" si="13"/>
+        <v>97340.415696020544</v>
       </c>
       <c r="K33" s="300">
-        <f t="shared" si="12"/>
-        <v>89179.291775760139</v>
+        <f t="shared" si="13"/>
+        <v>104387.89534596707</v>
       </c>
       <c r="M33" s="16" t="s">
         <v>98</v>
@@ -53725,11 +53764,11 @@
         <v>0.38200000000000001</v>
       </c>
       <c r="J37" s="299">
-        <f t="shared" ref="J37:K40" si="13">I37</f>
+        <f t="shared" ref="J37:K40" si="14">I37</f>
         <v>0.38200000000000001</v>
       </c>
       <c r="K37" s="299">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0.38200000000000001</v>
       </c>
       <c r="M37" t="s">
@@ -53768,11 +53807,11 @@
         <v>6.3E-2</v>
       </c>
       <c r="J38" s="299">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>6.3E-2</v>
       </c>
       <c r="K38" s="299">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>6.3E-2</v>
       </c>
       <c r="M38" t="s">
@@ -53811,11 +53850,11 @@
         <v>6.9000000000000006E-2</v>
       </c>
       <c r="J39" s="299">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>6.9000000000000006E-2</v>
       </c>
       <c r="K39" s="299">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>6.9000000000000006E-2</v>
       </c>
       <c r="M39" t="s">
@@ -53854,11 +53893,11 @@
         <v>0.16900000000000001</v>
       </c>
       <c r="J40" s="299">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0.16900000000000001</v>
       </c>
       <c r="K40" s="299">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0.16900000000000001</v>
       </c>
       <c r="M40" t="s">
@@ -53898,31 +53937,31 @@
       </c>
       <c r="D43" s="23"/>
       <c r="E43" s="23">
-        <f t="shared" ref="E43:K44" si="14">E14</f>
+        <f t="shared" ref="E43:K44" si="15">E14</f>
         <v>2017</v>
       </c>
       <c r="F43" s="23">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2018</v>
       </c>
       <c r="G43" s="24">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2019</v>
       </c>
       <c r="H43" s="24">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2020</v>
       </c>
       <c r="I43" s="24">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2021</v>
       </c>
       <c r="J43" s="24">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2022</v>
       </c>
       <c r="K43" s="24">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2023</v>
       </c>
     </row>
@@ -53933,31 +53972,31 @@
       </c>
       <c r="D44" s="25"/>
       <c r="E44" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>43008</v>
       </c>
       <c r="F44" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>43372</v>
       </c>
       <c r="G44" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>43738</v>
       </c>
       <c r="H44" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>44104</v>
       </c>
       <c r="I44" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>44469</v>
       </c>
       <c r="J44" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>44834</v>
       </c>
       <c r="K44" s="25">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>45199</v>
       </c>
     </row>
@@ -53974,11 +54013,26 @@
         <f>25913+40388+170799</f>
         <v>237100</v>
       </c>
-      <c r="G45" s="101"/>
-      <c r="H45" s="101"/>
-      <c r="I45" s="101"/>
-      <c r="J45" s="101"/>
-      <c r="K45" s="101"/>
+      <c r="G45" s="298">
+        <f>G90+F45</f>
+        <v>300609.96712000988</v>
+      </c>
+      <c r="H45" s="298">
+        <f t="shared" ref="H45:K45" si="16">H90+G45</f>
+        <v>374579.51445339958</v>
+      </c>
+      <c r="I45" s="298">
+        <f t="shared" si="16"/>
+        <v>454939.44004868198</v>
+      </c>
+      <c r="J45" s="298">
+        <f t="shared" si="16"/>
+        <v>541270.73842356959</v>
+      </c>
+      <c r="K45" s="298">
+        <f t="shared" si="16"/>
+        <v>633915.17385224556</v>
+      </c>
       <c r="M45" t="s">
         <v>118</v>
       </c>
@@ -53995,24 +54049,24 @@
         <v>23186</v>
       </c>
       <c r="G46" s="59">
-        <f>F46+ (1+G36)</f>
-        <v>23186.959999999999</v>
+        <f>F46* (1+G36)</f>
+        <v>22258.559999999998</v>
       </c>
       <c r="H46" s="59">
-        <f t="shared" ref="H46:K46" si="15">G46+ (1+H36)</f>
-        <v>23188.02</v>
+        <f t="shared" ref="H46:K46" si="17">G46* (1+H36)</f>
+        <v>23594.0736</v>
       </c>
       <c r="I46" s="59">
-        <f t="shared" si="15"/>
-        <v>23189.089</v>
+        <f t="shared" si="17"/>
+        <v>25222.064678399998</v>
       </c>
       <c r="J46" s="59">
-        <f t="shared" si="15"/>
-        <v>23190.157999999999</v>
+        <f t="shared" si="17"/>
+        <v>26962.387141209598</v>
       </c>
       <c r="K46" s="59">
-        <f t="shared" si="15"/>
-        <v>23191.226999999999</v>
+        <f t="shared" si="17"/>
+        <v>28822.791853953058</v>
       </c>
       <c r="M46" t="s">
         <v>103</v>
@@ -54034,19 +54088,19 @@
         <v>3831.2507254598308</v>
       </c>
       <c r="H47" s="59">
-        <f t="shared" ref="H47:K47" si="16">G47*(((H18/G18)))</f>
+        <f t="shared" ref="H47:K47" si="18">G47*(((H18/G18)))</f>
         <v>4041.5383456643308</v>
       </c>
       <c r="I47" s="59">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>4313.4248396710418</v>
       </c>
       <c r="J47" s="59">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>4611.0511536083422</v>
       </c>
       <c r="K47" s="59">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>4929.2136832073174</v>
       </c>
       <c r="M47" t="s">
@@ -54067,24 +54121,24 @@
         <v>37896</v>
       </c>
       <c r="G48" s="59">
-        <f>F48+(1+G36)</f>
-        <v>37896.959999999999</v>
+        <f>F48*(1+G36)</f>
+        <v>36380.159999999996</v>
       </c>
       <c r="H48" s="59">
-        <f t="shared" ref="H48:K48" si="17">G48+(1+H36)</f>
-        <v>37898.019999999997</v>
+        <f t="shared" ref="H48:K48" si="19">G48*(1+H36)</f>
+        <v>38562.969599999997</v>
       </c>
       <c r="I48" s="59">
-        <f t="shared" si="17"/>
-        <v>37899.089</v>
+        <f t="shared" si="19"/>
+        <v>41223.814502399997</v>
       </c>
       <c r="J48" s="59">
-        <f t="shared" si="17"/>
-        <v>37900.158000000003</v>
+        <f t="shared" si="19"/>
+        <v>44068.257703065596</v>
       </c>
       <c r="K48" s="59">
-        <f t="shared" si="17"/>
-        <v>37901.227000000006</v>
+        <f t="shared" si="19"/>
+        <v>47108.967484577122</v>
       </c>
       <c r="M48" t="s">
         <v>103</v>
@@ -54122,24 +54176,24 @@
         <v>22283</v>
       </c>
       <c r="G50" s="59">
-        <f>F50+(1+G36)</f>
-        <v>22283.96</v>
+        <f>F50*(1+G36)</f>
+        <v>21391.68</v>
       </c>
       <c r="H50" s="59">
-        <f t="shared" ref="H50:K50" si="18">G50+(1+H36)</f>
-        <v>22285.02</v>
+        <f t="shared" ref="H50:K50" si="20">G50*(1+H36)</f>
+        <v>22675.180800000002</v>
       </c>
       <c r="I50" s="59">
-        <f t="shared" si="18"/>
-        <v>22286.089</v>
+        <f t="shared" si="20"/>
+        <v>24239.7682752</v>
       </c>
       <c r="J50" s="59">
-        <f t="shared" si="18"/>
-        <v>22287.157999999999</v>
+        <f t="shared" si="20"/>
+        <v>25912.3122861888</v>
       </c>
       <c r="K50" s="59">
-        <f t="shared" si="18"/>
-        <v>22288.226999999999</v>
+        <f t="shared" si="20"/>
+        <v>27700.261833935827</v>
       </c>
       <c r="M50" t="s">
         <v>103</v>
@@ -54160,23 +54214,23 @@
       </c>
       <c r="G51" s="300">
         <f>SUM(G45:G50)</f>
-        <v>87199.130725459836</v>
+        <v>384471.61784546968</v>
       </c>
       <c r="H51" s="300">
-        <f t="shared" ref="H51:K51" si="19">SUM(H45:H50)</f>
-        <v>87412.59834566433</v>
+        <f t="shared" ref="H51:K51" si="21">SUM(H45:H50)</f>
+        <v>463453.2767990639</v>
       </c>
       <c r="I51" s="300">
-        <f t="shared" si="19"/>
-        <v>87687.691839671053</v>
+        <f t="shared" si="21"/>
+        <v>549938.51234435302</v>
       </c>
       <c r="J51" s="300">
-        <f t="shared" si="19"/>
-        <v>87988.525153608338</v>
+        <f t="shared" si="21"/>
+        <v>642824.74670764199</v>
       </c>
       <c r="K51" s="300">
-        <f t="shared" si="19"/>
-        <v>88309.894683207312</v>
+        <f t="shared" si="21"/>
+        <v>742476.40870791883</v>
       </c>
     </row>
     <row r="52" spans="3:13">
@@ -54201,19 +54255,19 @@
         <v>54125.616922269721</v>
       </c>
       <c r="H53" s="59">
-        <f t="shared" ref="H53:K53" si="20">G53*(H18/G18)</f>
+        <f t="shared" ref="H53:K53" si="22">G53*(H18/G18)</f>
         <v>57096.434545623888</v>
       </c>
       <c r="I53" s="59">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>60937.48418592901</v>
       </c>
       <c r="J53" s="59">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>65142.170594758092</v>
       </c>
       <c r="K53" s="59">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>69636.980365796393</v>
       </c>
       <c r="M53" t="s">
@@ -54236,19 +54290,19 @@
         <v>31379.52</v>
       </c>
       <c r="H54" s="59">
-        <f t="shared" ref="H54:K54" si="21">G54*(1+H36)</f>
+        <f t="shared" ref="H54:K54" si="23">G54*(1+H36)</f>
         <v>33262.2912</v>
       </c>
       <c r="I54" s="59">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>35557.389292799999</v>
       </c>
       <c r="J54" s="59">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>38010.849154003197</v>
       </c>
       <c r="K54" s="59">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>40633.597745629413</v>
       </c>
       <c r="M54" t="s">
@@ -54273,19 +54327,19 @@
         <v>9926.4</v>
       </c>
       <c r="H55" s="59">
-        <f t="shared" ref="H55:K55" si="22">G55*(1+H36)</f>
+        <f t="shared" ref="H55:K55" si="24">G55*(1+H36)</f>
         <v>10521.984</v>
       </c>
       <c r="I55" s="59">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>11248.000896</v>
       </c>
       <c r="J55" s="59">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>12024.112957824</v>
       </c>
       <c r="K55" s="59">
-        <f t="shared" si="22"/>
+        <f t="shared" si="24"/>
         <v>12853.776751913854</v>
       </c>
       <c r="M55" t="s">
@@ -54330,19 +54384,19 @@
         <v>102519</v>
       </c>
       <c r="H57" s="59">
-        <f t="shared" ref="H57:K57" si="23">$F$57</f>
+        <f t="shared" ref="H57:K57" si="25">$F$57</f>
         <v>102519</v>
       </c>
       <c r="I57" s="59">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>102519</v>
       </c>
       <c r="J57" s="59">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>102519</v>
       </c>
       <c r="K57" s="59">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>102519</v>
       </c>
       <c r="M57" t="s">
@@ -54361,24 +54415,24 @@
         <v>45180</v>
       </c>
       <c r="G58" s="59">
-        <f>F58+(1+G36)</f>
-        <v>45180.959999999999</v>
+        <f>F58*(1+G36)</f>
+        <v>43372.799999999996</v>
       </c>
       <c r="H58" s="59">
-        <f t="shared" ref="H58:K58" si="24">G58+(1+H36)</f>
-        <v>45182.02</v>
+        <f t="shared" ref="H58:K58" si="26">G58*(1+H36)</f>
+        <v>45975.167999999998</v>
       </c>
       <c r="I58" s="59">
-        <f t="shared" si="24"/>
-        <v>45183.089</v>
+        <f t="shared" si="26"/>
+        <v>49147.454591999995</v>
       </c>
       <c r="J58" s="59">
-        <f t="shared" si="24"/>
-        <v>45184.158000000003</v>
+        <f t="shared" si="26"/>
+        <v>52538.628958847992</v>
       </c>
       <c r="K58" s="59">
-        <f t="shared" si="24"/>
-        <v>45185.227000000006</v>
+        <f t="shared" si="26"/>
+        <v>56163.794357008504</v>
       </c>
       <c r="M58" t="s">
         <v>103</v>
@@ -54399,23 +54453,23 @@
       </c>
       <c r="G59" s="59">
         <f>SUM(G53:G58)</f>
-        <v>243131.49692226973</v>
+        <v>241323.33692226972</v>
       </c>
       <c r="H59" s="59">
-        <f t="shared" ref="H59:K59" si="25">SUM(H53:H58)</f>
-        <v>248581.72974562386</v>
+        <f t="shared" ref="H59:K59" si="27">SUM(H53:H58)</f>
+        <v>249374.87774562387</v>
       </c>
       <c r="I59" s="59">
-        <f t="shared" si="25"/>
-        <v>255444.96337472901</v>
+        <f t="shared" si="27"/>
+        <v>259409.32896672899</v>
       </c>
       <c r="J59" s="59">
-        <f t="shared" si="25"/>
-        <v>262880.29070658528</v>
+        <f t="shared" si="27"/>
+        <v>270234.7616654333</v>
       </c>
       <c r="K59" s="59">
-        <f t="shared" si="25"/>
-        <v>270828.58186333964</v>
+        <f t="shared" si="27"/>
+        <v>281807.14922034816</v>
       </c>
     </row>
     <row r="60" spans="3:13">
@@ -54435,11 +54489,26 @@
       <c r="F61" s="3">
         <v>40201</v>
       </c>
-      <c r="G61" s="101"/>
-      <c r="H61" s="101"/>
-      <c r="I61" s="101"/>
-      <c r="J61" s="101"/>
-      <c r="K61" s="101"/>
+      <c r="G61" s="59">
+        <f>F61+G32</f>
+        <v>45327.4</v>
+      </c>
+      <c r="H61" s="59">
+        <f t="shared" ref="H61:K61" si="28">G61+H32</f>
+        <v>50761.383999999998</v>
+      </c>
+      <c r="I61" s="59">
+        <f t="shared" si="28"/>
+        <v>56570.312895999996</v>
+      </c>
+      <c r="J61" s="59">
+        <f t="shared" si="28"/>
+        <v>62780.057885823997</v>
+      </c>
+      <c r="K61" s="59">
+        <f t="shared" si="28"/>
+        <v>69418.275279945854</v>
+      </c>
       <c r="M61" t="s">
         <v>154</v>
       </c>
@@ -54475,11 +54544,26 @@
       <c r="F63" s="3">
         <v>-3454</v>
       </c>
-      <c r="G63" s="101"/>
-      <c r="H63" s="101"/>
-      <c r="I63" s="101"/>
-      <c r="J63" s="101"/>
-      <c r="K63" s="101"/>
+      <c r="G63" s="59">
+        <f>$F$63</f>
+        <v>-3454</v>
+      </c>
+      <c r="H63" s="59">
+        <f t="shared" ref="H63:K63" si="29">$F$63</f>
+        <v>-3454</v>
+      </c>
+      <c r="I63" s="59">
+        <f t="shared" si="29"/>
+        <v>-3454</v>
+      </c>
+      <c r="J63" s="59">
+        <f t="shared" si="29"/>
+        <v>-3454</v>
+      </c>
+      <c r="K63" s="59">
+        <f t="shared" si="29"/>
+        <v>-3454</v>
+      </c>
       <c r="M63" t="s">
         <v>100</v>
       </c>
@@ -54497,52 +54581,67 @@
         <f>SUM(F61:F63)</f>
         <v>107147</v>
       </c>
-      <c r="G64" s="228"/>
-      <c r="H64" s="228"/>
-      <c r="I64" s="228"/>
-      <c r="J64" s="228"/>
-      <c r="K64" s="228"/>
-    </row>
-    <row r="65" spans="2:13">
+      <c r="G64" s="102">
+        <f>SUM(G61:G63)</f>
+        <v>41873.4</v>
+      </c>
+      <c r="H64" s="102">
+        <f t="shared" ref="H64:K64" si="30">SUM(H61:H63)</f>
+        <v>47307.383999999998</v>
+      </c>
+      <c r="I64" s="102">
+        <f t="shared" si="30"/>
+        <v>53116.312895999996</v>
+      </c>
+      <c r="J64" s="102">
+        <f t="shared" si="30"/>
+        <v>59326.057885823997</v>
+      </c>
+      <c r="K64" s="102">
+        <f t="shared" si="30"/>
+        <v>65964.275279945854</v>
+      </c>
+    </row>
+    <row r="65" spans="2:14">
       <c r="D65" s="18"/>
       <c r="E65" s="18"/>
       <c r="F65" s="18"/>
     </row>
-    <row r="66" spans="2:13">
+    <row r="66" spans="2:14">
       <c r="C66" s="12" t="s">
         <v>26</v>
       </c>
       <c r="D66" s="30"/>
       <c r="E66" s="30">
-        <f t="shared" ref="E66:K66" si="26">ROUND(E51-E59-E64,3)</f>
+        <f t="shared" ref="E66:G66" si="31">ROUND(E51-E59-E64,3)</f>
         <v>0</v>
       </c>
       <c r="F66" s="30">
-        <f t="shared" si="26"/>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="G66" s="30">
-        <f t="shared" si="26"/>
-        <v>-155932.36600000001</v>
+        <f t="shared" si="31"/>
+        <v>101274.88099999999</v>
       </c>
       <c r="H66" s="30">
-        <f t="shared" si="26"/>
-        <v>-161169.13099999999</v>
+        <f t="shared" ref="H66:K66" si="32">ROUND(H51-H59-H64,3)</f>
+        <v>166771.01500000001</v>
       </c>
       <c r="I66" s="30">
-        <f t="shared" si="26"/>
-        <v>-167757.272</v>
+        <f t="shared" si="32"/>
+        <v>237412.87</v>
       </c>
       <c r="J66" s="30">
-        <f t="shared" si="26"/>
-        <v>-174891.766</v>
+        <f t="shared" si="32"/>
+        <v>313263.92700000003</v>
       </c>
       <c r="K66" s="30">
-        <f t="shared" si="26"/>
-        <v>-182518.68700000001</v>
-      </c>
-    </row>
-    <row r="67" spans="2:13">
+        <f t="shared" si="32"/>
+        <v>394704.984</v>
+      </c>
+    </row>
+    <row r="67" spans="2:14">
       <c r="E67" s="18"/>
       <c r="F67" s="18"/>
       <c r="H67" s="18"/>
@@ -54550,7 +54649,7 @@
       <c r="J67" s="18"/>
       <c r="K67" s="18"/>
     </row>
-    <row r="68" spans="2:13">
+    <row r="68" spans="2:14">
       <c r="B68" t="s">
         <v>316</v>
       </c>
@@ -54566,7 +54665,7 @@
       <c r="J68" s="11"/>
       <c r="K68" s="11"/>
     </row>
-    <row r="69" spans="2:13">
+    <row r="69" spans="2:14">
       <c r="C69" s="26" t="str">
         <f>C14</f>
         <v xml:space="preserve">Fiscal year  </v>
@@ -54575,27 +54674,27 @@
       <c r="E69" s="23"/>
       <c r="F69" s="23"/>
       <c r="G69" s="24">
-        <f t="shared" ref="G69:K70" si="27">G14</f>
+        <f t="shared" ref="G69:K70" si="33">G14</f>
         <v>2019</v>
       </c>
       <c r="H69" s="24">
-        <f t="shared" si="27"/>
+        <f t="shared" si="33"/>
         <v>2020</v>
       </c>
       <c r="I69" s="24">
-        <f t="shared" si="27"/>
+        <f t="shared" si="33"/>
         <v>2021</v>
       </c>
       <c r="J69" s="24">
-        <f t="shared" si="27"/>
+        <f t="shared" si="33"/>
         <v>2022</v>
       </c>
       <c r="K69" s="24">
-        <f t="shared" si="27"/>
+        <f t="shared" si="33"/>
         <v>2023</v>
       </c>
     </row>
-    <row r="70" spans="2:13">
+    <row r="70" spans="2:14">
       <c r="C70" s="7" t="str">
         <f>C15</f>
         <v>Fiscal year end date</v>
@@ -54604,27 +54703,27 @@
       <c r="E70" s="25"/>
       <c r="F70" s="25"/>
       <c r="G70" s="25">
-        <f t="shared" si="27"/>
+        <f t="shared" si="33"/>
         <v>43738</v>
       </c>
       <c r="H70" s="25">
-        <f t="shared" si="27"/>
+        <f t="shared" si="33"/>
         <v>44104</v>
       </c>
       <c r="I70" s="25">
-        <f t="shared" si="27"/>
+        <f t="shared" si="33"/>
         <v>44469</v>
       </c>
       <c r="J70" s="25">
-        <f t="shared" si="27"/>
+        <f t="shared" si="33"/>
         <v>44834</v>
       </c>
       <c r="K70" s="25">
-        <f t="shared" si="27"/>
+        <f t="shared" si="33"/>
         <v>45199</v>
       </c>
     </row>
-    <row r="72" spans="2:13">
+    <row r="72" spans="2:14">
       <c r="C72" t="s">
         <v>2</v>
       </c>
@@ -54636,52 +54735,52 @@
         <v>51031.271323199988</v>
       </c>
       <c r="H72" s="298">
-        <f t="shared" ref="H72:K72" si="28">H28</f>
+        <f t="shared" ref="H72:K72" si="34">H28</f>
         <v>55490.56177824</v>
       </c>
       <c r="I72" s="298">
-        <f t="shared" si="28"/>
+        <f t="shared" si="34"/>
         <v>59656.257121751987</v>
       </c>
       <c r="J72" s="298">
-        <f t="shared" si="28"/>
+        <f t="shared" si="34"/>
         <v>63797.825362152886</v>
       </c>
       <c r="K72" s="298">
-        <f t="shared" si="28"/>
+        <f t="shared" si="34"/>
         <v>68225.161811141414</v>
       </c>
       <c r="M72" s="16"/>
     </row>
-    <row r="73" spans="2:13">
+    <row r="73" spans="2:14">
       <c r="C73" t="s">
         <v>33</v>
       </c>
       <c r="D73" s="34"/>
       <c r="E73" s="34"/>
       <c r="F73" s="34"/>
-      <c r="G73" s="105">
-        <f>G30</f>
-        <v>0</v>
-      </c>
-      <c r="H73" s="105">
-        <f t="shared" ref="H73:K73" si="29">H30</f>
-        <v>0</v>
-      </c>
-      <c r="I73" s="105">
-        <f t="shared" si="29"/>
-        <v>0</v>
-      </c>
-      <c r="J73" s="105">
-        <f t="shared" si="29"/>
-        <v>0</v>
-      </c>
-      <c r="K73" s="105">
-        <f t="shared" si="29"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="2:13">
+      <c r="G73" s="304">
+        <f>G106</f>
+        <v>10722.489599999999</v>
+      </c>
+      <c r="H73" s="304">
+        <f t="shared" ref="H73:K73" si="35">H106</f>
+        <v>11636.785152</v>
+      </c>
+      <c r="I73" s="304">
+        <f t="shared" si="35"/>
+        <v>12729.364789632</v>
+      </c>
+      <c r="J73" s="304">
+        <f t="shared" si="35"/>
+        <v>13917.317683148543</v>
+      </c>
+      <c r="K73" s="304">
+        <f t="shared" si="35"/>
+        <v>15208.603570206933</v>
+      </c>
+    </row>
+    <row r="74" spans="2:14">
       <c r="C74" t="s">
         <v>74</v>
       </c>
@@ -54693,83 +54792,163 @@
         <v>5126.3999999999996</v>
       </c>
       <c r="H74" s="59">
-        <f t="shared" ref="H74:K74" si="30">H32</f>
+        <f t="shared" ref="H74:K74" si="36">H32</f>
         <v>5433.9839999999995</v>
       </c>
       <c r="I74" s="59">
-        <f t="shared" si="30"/>
+        <f t="shared" si="36"/>
         <v>5808.9288959999994</v>
       </c>
       <c r="J74" s="59">
-        <f t="shared" si="30"/>
+        <f t="shared" si="36"/>
         <v>6209.7449898239993</v>
       </c>
       <c r="K74" s="59">
-        <f t="shared" si="30"/>
+        <f t="shared" si="36"/>
         <v>6638.2173941218552</v>
       </c>
     </row>
-    <row r="75" spans="2:13">
+    <row r="75" spans="2:14">
       <c r="C75" t="s">
         <v>65</v>
       </c>
       <c r="D75" s="18"/>
       <c r="E75" s="18"/>
       <c r="F75" s="18"/>
-      <c r="G75" s="101"/>
-      <c r="H75" s="101"/>
-      <c r="I75" s="101"/>
-      <c r="J75" s="101"/>
-      <c r="K75" s="101"/>
-    </row>
-    <row r="76" spans="2:13">
+      <c r="G75" s="59">
+        <f>SUM(F46:F48) - SUM(G46:G48)</f>
+        <v>2568.0292745401748</v>
+      </c>
+      <c r="H75" s="59">
+        <f>SUM(G46:G48) - SUM(H46:H48)</f>
+        <v>-3728.610820204507</v>
+      </c>
+      <c r="I75" s="59">
+        <f t="shared" ref="I75:K75" si="37">SUM(H46:H48) - SUM(I46:I48)</f>
+        <v>-4560.7224748067092</v>
+      </c>
+      <c r="J75" s="59">
+        <f t="shared" si="37"/>
+        <v>-4882.3919774124952</v>
+      </c>
+      <c r="K75" s="59">
+        <f t="shared" si="37"/>
+        <v>-5219.277023853967</v>
+      </c>
+    </row>
+    <row r="76" spans="2:14">
       <c r="C76" t="s">
         <v>66</v>
       </c>
       <c r="D76" s="18"/>
       <c r="E76" s="18"/>
       <c r="F76" s="18"/>
-      <c r="G76" s="101"/>
-      <c r="H76" s="101"/>
-      <c r="I76" s="101"/>
-      <c r="J76" s="101"/>
-      <c r="K76" s="101"/>
-    </row>
-    <row r="77" spans="2:13">
+      <c r="G76" s="59">
+        <f>-(SUM(F53:F55) - SUM(G53:G55))</f>
+        <v>-3483.4630777302809</v>
+      </c>
+      <c r="H76" s="59">
+        <f t="shared" ref="H76:K76" si="38">-(SUM(G53:G55) - SUM(H53:H55))</f>
+        <v>5449.1728233541653</v>
+      </c>
+      <c r="I76" s="59">
+        <f t="shared" si="38"/>
+        <v>6862.1646291051293</v>
+      </c>
+      <c r="J76" s="59">
+        <f t="shared" si="38"/>
+        <v>7434.2583318562683</v>
+      </c>
+      <c r="K76" s="59">
+        <f t="shared" si="38"/>
+        <v>7947.2221567543747</v>
+      </c>
+    </row>
+    <row r="77" spans="2:14">
       <c r="C77" t="s">
         <v>56</v>
       </c>
-      <c r="G77" s="96"/>
-      <c r="H77" s="96"/>
-      <c r="I77" s="96"/>
-      <c r="J77" s="96"/>
-      <c r="K77" s="96"/>
-      <c r="M77" t="s">
+      <c r="G77" s="304">
+        <f>G111</f>
+        <v>-647.56000000000131</v>
+      </c>
+      <c r="H77" s="304">
+        <f t="shared" ref="H77:K77" si="39">H111</f>
+        <v>-2914.7136000000028</v>
+      </c>
+      <c r="I77" s="304">
+        <f t="shared" si="39"/>
+        <v>-3308.3539583999991</v>
+      </c>
+      <c r="J77" s="304">
+        <f t="shared" si="39"/>
+        <v>-3536.6303815296014</v>
+      </c>
+      <c r="K77" s="304">
+        <f t="shared" si="39"/>
+        <v>-3780.6578778551411</v>
+      </c>
+      <c r="M77" s="16" t="s">
+        <v>333</v>
+      </c>
+      <c r="N77" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="78" spans="2:13">
+    <row r="78" spans="2:14">
       <c r="C78" t="s">
         <v>59</v>
       </c>
-      <c r="G78" s="101"/>
-      <c r="H78" s="101"/>
-      <c r="I78" s="101"/>
-      <c r="J78" s="101"/>
-      <c r="K78" s="101"/>
-      <c r="M78" s="16"/>
-    </row>
-    <row r="79" spans="2:13">
+      <c r="G78" s="59">
+        <f>G58-F58</f>
+        <v>-1807.2000000000044</v>
+      </c>
+      <c r="H78" s="59">
+        <f t="shared" ref="H78:K78" si="40">H58-G58</f>
+        <v>2602.3680000000022</v>
+      </c>
+      <c r="I78" s="59">
+        <f t="shared" si="40"/>
+        <v>3172.2865919999967</v>
+      </c>
+      <c r="J78" s="59">
+        <f t="shared" si="40"/>
+        <v>3391.1743668479976</v>
+      </c>
+      <c r="K78" s="59">
+        <f t="shared" si="40"/>
+        <v>3625.1653981605123</v>
+      </c>
+      <c r="M78" s="16" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="79" spans="2:14">
       <c r="C79" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="G79" s="228"/>
-      <c r="H79" s="228"/>
-      <c r="I79" s="228"/>
-      <c r="J79" s="228"/>
-      <c r="K79" s="228"/>
-    </row>
-    <row r="81" spans="3:13">
+      <c r="G79" s="300">
+        <f>SUM(G72:G78)</f>
+        <v>63509.967120009875</v>
+      </c>
+      <c r="H79" s="300">
+        <f t="shared" ref="H79:K79" si="41">SUM(H72:H78)</f>
+        <v>73969.547333389666</v>
+      </c>
+      <c r="I79" s="300">
+        <f t="shared" si="41"/>
+        <v>80359.925595282402</v>
+      </c>
+      <c r="J79" s="300">
+        <f t="shared" si="41"/>
+        <v>86331.298374887614</v>
+      </c>
+      <c r="K79" s="300">
+        <f t="shared" si="41"/>
+        <v>92644.435428675992</v>
+      </c>
+    </row>
+    <row r="81" spans="2:13">
       <c r="C81" t="s">
         <v>35</v>
       </c>
@@ -54779,17 +54958,32 @@
       <c r="J81" s="96"/>
       <c r="K81" s="96"/>
     </row>
-    <row r="82" spans="3:13">
+    <row r="82" spans="2:13">
       <c r="C82" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="G82" s="228"/>
-      <c r="H82" s="228"/>
-      <c r="I82" s="228"/>
-      <c r="J82" s="228"/>
-      <c r="K82" s="228"/>
-    </row>
-    <row r="84" spans="3:13">
+      <c r="G82" s="228">
+        <f>SUM(G81)</f>
+        <v>0</v>
+      </c>
+      <c r="H82" s="228">
+        <f t="shared" ref="H82:K82" si="42">SUM(H81)</f>
+        <v>0</v>
+      </c>
+      <c r="I82" s="228">
+        <f t="shared" si="42"/>
+        <v>0</v>
+      </c>
+      <c r="J82" s="228">
+        <f t="shared" si="42"/>
+        <v>0</v>
+      </c>
+      <c r="K82" s="228">
+        <f t="shared" si="42"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="2:13">
       <c r="C84" t="s">
         <v>67</v>
       </c>
@@ -54799,57 +54993,90 @@
       <c r="J84" s="97"/>
       <c r="K84" s="97"/>
     </row>
-    <row r="85" spans="3:13">
+    <row r="85" spans="2:13">
       <c r="C85" t="s">
         <v>23</v>
       </c>
-      <c r="G85" s="96"/>
-      <c r="H85" s="96"/>
-      <c r="I85" s="96"/>
-      <c r="J85" s="96"/>
-      <c r="K85" s="96"/>
-    </row>
-    <row r="86" spans="3:13">
+      <c r="G85" s="302"/>
+      <c r="H85" s="302"/>
+      <c r="I85" s="302"/>
+      <c r="J85" s="302"/>
+      <c r="K85" s="302"/>
+    </row>
+    <row r="86" spans="2:13">
       <c r="C86" t="s">
         <v>70</v>
       </c>
-      <c r="G86" s="96"/>
-      <c r="H86" s="96"/>
-      <c r="I86" s="96"/>
-      <c r="J86" s="96"/>
-      <c r="K86" s="96"/>
-    </row>
-    <row r="87" spans="3:13">
+      <c r="G86" s="302"/>
+      <c r="H86" s="302"/>
+      <c r="I86" s="302"/>
+      <c r="J86" s="302"/>
+      <c r="K86" s="302"/>
+    </row>
+    <row r="87" spans="2:13">
       <c r="C87" t="s">
         <v>71</v>
       </c>
-      <c r="G87" s="96"/>
-      <c r="H87" s="96"/>
-      <c r="I87" s="96"/>
-      <c r="J87" s="96"/>
-      <c r="K87" s="96"/>
-    </row>
-    <row r="88" spans="3:13">
+      <c r="G87" s="302"/>
+      <c r="H87" s="302"/>
+      <c r="I87" s="302"/>
+      <c r="J87" s="302"/>
+      <c r="K87" s="302"/>
+    </row>
+    <row r="88" spans="2:13">
       <c r="C88" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="G88" s="228"/>
-      <c r="H88" s="228"/>
-      <c r="I88" s="228"/>
-      <c r="J88" s="228"/>
-      <c r="K88" s="228"/>
-    </row>
-    <row r="90" spans="3:13">
+      <c r="G88" s="228">
+        <f>SUM(G84:G87)</f>
+        <v>0</v>
+      </c>
+      <c r="H88" s="228">
+        <f t="shared" ref="H88:K88" si="43">SUM(H84:H87)</f>
+        <v>0</v>
+      </c>
+      <c r="I88" s="228">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="J88" s="228">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="K88" s="228">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="2:13">
       <c r="C90" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="G90" s="228"/>
-      <c r="H90" s="228"/>
-      <c r="I90" s="228"/>
-      <c r="J90" s="228"/>
-      <c r="K90" s="228"/>
-    </row>
-    <row r="92" spans="3:13">
+      <c r="G90" s="300">
+        <f>G88+G82+G79</f>
+        <v>63509.967120009875</v>
+      </c>
+      <c r="H90" s="300">
+        <f t="shared" ref="H90:K90" si="44">H88+H82+H79</f>
+        <v>73969.547333389666</v>
+      </c>
+      <c r="I90" s="300">
+        <f t="shared" si="44"/>
+        <v>80359.925595282402</v>
+      </c>
+      <c r="J90" s="300">
+        <f t="shared" si="44"/>
+        <v>86331.298374887614</v>
+      </c>
+      <c r="K90" s="300">
+        <f t="shared" si="44"/>
+        <v>92644.435428675992</v>
+      </c>
+    </row>
+    <row r="92" spans="2:13">
+      <c r="B92" t="s">
+        <v>316</v>
+      </c>
       <c r="C92" s="5" t="s">
         <v>29</v>
       </c>
@@ -54862,83 +55089,83 @@
       <c r="J92" s="7"/>
       <c r="K92" s="7"/>
     </row>
-    <row r="93" spans="3:13">
+    <row r="93" spans="2:13">
       <c r="C93" s="26" t="str">
-        <f t="shared" ref="C93:K93" si="31">C14</f>
+        <f t="shared" ref="C93:K93" si="45">C14</f>
         <v xml:space="preserve">Fiscal year  </v>
       </c>
       <c r="D93" s="23">
-        <f t="shared" si="31"/>
+        <f t="shared" si="45"/>
         <v>2016</v>
       </c>
       <c r="E93" s="23">
-        <f t="shared" si="31"/>
+        <f t="shared" si="45"/>
         <v>2017</v>
       </c>
       <c r="F93" s="23">
-        <f t="shared" si="31"/>
+        <f t="shared" si="45"/>
         <v>2018</v>
       </c>
       <c r="G93" s="24">
-        <f t="shared" si="31"/>
+        <f t="shared" si="45"/>
         <v>2019</v>
       </c>
       <c r="H93" s="24">
-        <f t="shared" si="31"/>
+        <f t="shared" si="45"/>
         <v>2020</v>
       </c>
       <c r="I93" s="24">
-        <f t="shared" si="31"/>
+        <f t="shared" si="45"/>
         <v>2021</v>
       </c>
       <c r="J93" s="24">
-        <f t="shared" si="31"/>
+        <f t="shared" si="45"/>
         <v>2022</v>
       </c>
       <c r="K93" s="24">
-        <f t="shared" si="31"/>
+        <f t="shared" si="45"/>
         <v>2023</v>
       </c>
     </row>
-    <row r="94" spans="3:13">
+    <row r="94" spans="2:13">
       <c r="C94" s="7" t="str">
-        <f t="shared" ref="C94:K94" si="32">C15</f>
+        <f t="shared" ref="C94:K94" si="46">C15</f>
         <v>Fiscal year end date</v>
       </c>
       <c r="D94" s="25">
-        <f t="shared" si="32"/>
+        <f t="shared" si="46"/>
         <v>42643</v>
       </c>
       <c r="E94" s="25">
-        <f t="shared" si="32"/>
+        <f t="shared" si="46"/>
         <v>43008</v>
       </c>
       <c r="F94" s="25">
-        <f t="shared" si="32"/>
+        <f t="shared" si="46"/>
         <v>43372</v>
       </c>
       <c r="G94" s="25">
-        <f t="shared" si="32"/>
+        <f t="shared" si="46"/>
         <v>43738</v>
       </c>
       <c r="H94" s="25">
-        <f t="shared" si="32"/>
+        <f t="shared" si="46"/>
         <v>44104</v>
       </c>
       <c r="I94" s="25">
-        <f t="shared" si="32"/>
+        <f t="shared" si="46"/>
         <v>44469</v>
       </c>
       <c r="J94" s="25">
-        <f t="shared" si="32"/>
+        <f t="shared" si="46"/>
         <v>44834</v>
       </c>
       <c r="K94" s="25">
-        <f t="shared" si="32"/>
+        <f t="shared" si="46"/>
         <v>45199</v>
       </c>
     </row>
-    <row r="95" spans="3:13">
+    <row r="95" spans="2:13">
       <c r="C95" s="16"/>
       <c r="G95" s="76" t="s">
         <v>116</v>
@@ -54948,15 +55175,30 @@
       <c r="J95" s="76"/>
       <c r="K95" s="76"/>
     </row>
-    <row r="96" spans="3:13">
+    <row r="96" spans="2:13">
       <c r="C96" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="G96" s="59"/>
-      <c r="H96" s="59"/>
-      <c r="I96" s="59"/>
-      <c r="J96" s="59"/>
-      <c r="K96" s="59"/>
+      <c r="G96" s="59">
+        <f>F99</f>
+        <v>41304</v>
+      </c>
+      <c r="H96" s="59">
+        <f t="shared" ref="H96:K96" si="47">G99</f>
+        <v>44900.8704</v>
+      </c>
+      <c r="I96" s="59">
+        <f t="shared" si="47"/>
+        <v>48442.606847999996</v>
+      </c>
+      <c r="J96" s="59">
+        <f t="shared" si="47"/>
+        <v>51939.081648767991</v>
+      </c>
+      <c r="K96" s="59">
+        <f t="shared" si="47"/>
+        <v>55367.186487757041</v>
+      </c>
       <c r="M96" t="s">
         <v>166</v>
       </c>
@@ -54975,19 +55217,27 @@
         <v>13313</v>
       </c>
       <c r="G97" s="3">
-        <v>13285</v>
+        <f>F97*(1+G36)</f>
+        <v>12780.48</v>
       </c>
       <c r="H97" s="3">
-        <v>13649</v>
+        <f t="shared" ref="H97:K97" si="48">G97*(1+H36)</f>
+        <v>13547.308800000001</v>
       </c>
       <c r="I97" s="3">
-        <v>13819</v>
+        <f t="shared" si="48"/>
+        <v>14482.0731072</v>
       </c>
       <c r="J97" s="3">
-        <v>14000</v>
+        <f t="shared" si="48"/>
+        <v>15481.336151596799</v>
       </c>
       <c r="K97" s="3">
-        <v>14200</v>
+        <f t="shared" si="48"/>
+        <v>16549.548346056978</v>
+      </c>
+      <c r="L97" s="303" t="s">
+        <v>334</v>
       </c>
       <c r="M97" t="s">
         <v>153</v>
@@ -55006,11 +55256,26 @@
       <c r="F98" s="62">
         <v>-9300</v>
       </c>
-      <c r="G98" s="103"/>
-      <c r="H98" s="103"/>
-      <c r="I98" s="103"/>
-      <c r="J98" s="103"/>
-      <c r="K98" s="103"/>
+      <c r="G98" s="103">
+        <f>(G101*G97) *-1</f>
+        <v>-9183.6095999999998</v>
+      </c>
+      <c r="H98" s="103">
+        <f t="shared" ref="H98:K98" si="49">(H101*H97) *-1</f>
+        <v>-10005.572352000001</v>
+      </c>
+      <c r="I98" s="103">
+        <f t="shared" si="49"/>
+        <v>-10985.598306432001</v>
+      </c>
+      <c r="J98" s="103">
+        <f t="shared" si="49"/>
+        <v>-12053.231312607744</v>
+      </c>
+      <c r="K98" s="103">
+        <f t="shared" si="49"/>
+        <v>-13215.895240098818</v>
+      </c>
       <c r="M98" t="s">
         <v>165</v>
       </c>
@@ -55028,11 +55293,26 @@
         <f>F49</f>
         <v>41304</v>
       </c>
-      <c r="G99" s="102"/>
-      <c r="H99" s="102"/>
-      <c r="I99" s="102"/>
-      <c r="J99" s="102"/>
-      <c r="K99" s="102"/>
+      <c r="G99" s="102">
+        <f>SUM(G96:G98)</f>
+        <v>44900.8704</v>
+      </c>
+      <c r="H99" s="102">
+        <f t="shared" ref="H99:K99" si="50">SUM(H96:H98)</f>
+        <v>48442.606847999996</v>
+      </c>
+      <c r="I99" s="102">
+        <f t="shared" si="50"/>
+        <v>51939.081648767991</v>
+      </c>
+      <c r="J99" s="102">
+        <f t="shared" si="50"/>
+        <v>55367.186487757041</v>
+      </c>
+      <c r="K99" s="102">
+        <f t="shared" si="50"/>
+        <v>58700.839593715194</v>
+      </c>
       <c r="M99" t="s">
         <v>164</v>
       </c>
@@ -55059,11 +55339,26 @@
         <f>-(F98/F97)</f>
         <v>0.69856531210095396</v>
       </c>
-      <c r="G101" s="95"/>
-      <c r="H101" s="95"/>
-      <c r="I101" s="95"/>
-      <c r="J101" s="95"/>
-      <c r="K101" s="95"/>
+      <c r="G101" s="95">
+        <f>F101+$M$101</f>
+        <v>0.71856531210095398</v>
+      </c>
+      <c r="H101" s="95">
+        <f t="shared" ref="H101:K101" si="51">G101+$M$101</f>
+        <v>0.738565312100954</v>
+      </c>
+      <c r="I101" s="95">
+        <f t="shared" si="51"/>
+        <v>0.75856531210095401</v>
+      </c>
+      <c r="J101" s="95">
+        <f>I101+$M$101</f>
+        <v>0.77856531210095403</v>
+      </c>
+      <c r="K101" s="95">
+        <f t="shared" si="51"/>
+        <v>0.79856531210095405</v>
+      </c>
       <c r="M101" s="55">
         <v>0.02</v>
       </c>
@@ -55114,11 +55409,26 @@
         <f>F106+F98</f>
         <v>1603</v>
       </c>
-      <c r="G104" s="99"/>
-      <c r="H104" s="99"/>
-      <c r="I104" s="99"/>
-      <c r="J104" s="99"/>
-      <c r="K104" s="99"/>
+      <c r="G104" s="99">
+        <f>G105*G17</f>
+        <v>1538.8799999999999</v>
+      </c>
+      <c r="H104" s="99">
+        <f t="shared" ref="H104:K104" si="52">H105*H17</f>
+        <v>1631.2128</v>
+      </c>
+      <c r="I104" s="99">
+        <f t="shared" si="52"/>
+        <v>1743.7664832</v>
+      </c>
+      <c r="J104" s="99">
+        <f t="shared" si="52"/>
+        <v>1864.0863705407999</v>
+      </c>
+      <c r="K104" s="99">
+        <f t="shared" si="52"/>
+        <v>1992.708330108115</v>
+      </c>
       <c r="M104" t="s">
         <v>237</v>
       </c>
@@ -55142,11 +55452,26 @@
         <f>F104/F17</f>
         <v>6.0355051864681188E-3</v>
       </c>
-      <c r="G105" s="95"/>
-      <c r="H105" s="95"/>
-      <c r="I105" s="95"/>
-      <c r="J105" s="95"/>
-      <c r="K105" s="95"/>
+      <c r="G105" s="95">
+        <f>$F$105</f>
+        <v>6.0355051864681188E-3</v>
+      </c>
+      <c r="H105" s="95">
+        <f t="shared" ref="H105:K105" si="53">$F$105</f>
+        <v>6.0355051864681188E-3</v>
+      </c>
+      <c r="I105" s="95">
+        <f t="shared" si="53"/>
+        <v>6.0355051864681188E-3</v>
+      </c>
+      <c r="J105" s="95">
+        <f t="shared" si="53"/>
+        <v>6.0355051864681188E-3</v>
+      </c>
+      <c r="K105" s="95">
+        <f t="shared" si="53"/>
+        <v>6.0355051864681188E-3</v>
+      </c>
       <c r="M105" t="s">
         <v>157</v>
       </c>
@@ -55170,11 +55495,26 @@
         <f>F30</f>
         <v>10903</v>
       </c>
-      <c r="G106" s="100"/>
-      <c r="H106" s="100"/>
-      <c r="I106" s="100"/>
-      <c r="J106" s="100"/>
-      <c r="K106" s="100"/>
+      <c r="G106" s="100">
+        <f>G104-G98</f>
+        <v>10722.489599999999</v>
+      </c>
+      <c r="H106" s="100">
+        <f t="shared" ref="H106:K106" si="54">H104-H98</f>
+        <v>11636.785152</v>
+      </c>
+      <c r="I106" s="100">
+        <f t="shared" si="54"/>
+        <v>12729.364789632</v>
+      </c>
+      <c r="J106" s="100">
+        <f t="shared" si="54"/>
+        <v>13917.317683148543</v>
+      </c>
+      <c r="K106" s="100">
+        <f t="shared" si="54"/>
+        <v>15208.603570206933</v>
+      </c>
       <c r="M106" t="s">
         <v>159</v>
       </c>
@@ -55205,11 +55545,26 @@
         <v>27</v>
       </c>
       <c r="D109" s="18"/>
-      <c r="G109" s="108"/>
-      <c r="H109" s="108"/>
-      <c r="I109" s="108"/>
-      <c r="J109" s="108"/>
-      <c r="K109" s="108"/>
+      <c r="G109" s="108">
+        <f>F112</f>
+        <v>22283</v>
+      </c>
+      <c r="H109" s="108">
+        <f t="shared" ref="H109:K109" si="55">G112</f>
+        <v>21391.68</v>
+      </c>
+      <c r="I109" s="108">
+        <f t="shared" si="55"/>
+        <v>22675.180800000002</v>
+      </c>
+      <c r="J109" s="108">
+        <f t="shared" si="55"/>
+        <v>24239.7682752</v>
+      </c>
+      <c r="K109" s="108">
+        <f t="shared" si="55"/>
+        <v>25912.3122861888</v>
+      </c>
       <c r="M109" t="s">
         <v>166</v>
       </c>
@@ -55220,23 +55575,23 @@
       </c>
       <c r="G110" s="18">
         <f>-(G104)</f>
-        <v>0</v>
+        <v>-1538.8799999999999</v>
       </c>
       <c r="H110" s="18">
         <f>-(H104)</f>
-        <v>0</v>
+        <v>-1631.2128</v>
       </c>
       <c r="I110" s="18">
         <f>-(I104)</f>
-        <v>0</v>
+        <v>-1743.7664832</v>
       </c>
       <c r="J110" s="18">
         <f>-(J104)</f>
-        <v>0</v>
+        <v>-1864.0863705407999</v>
       </c>
       <c r="K110" s="18">
         <f>-(K104)</f>
-        <v>0</v>
+        <v>-1992.708330108115</v>
       </c>
       <c r="M110" t="s">
         <v>161</v>
@@ -55249,11 +55604,26 @@
       <c r="D111" s="67"/>
       <c r="E111" s="67"/>
       <c r="F111" s="67"/>
-      <c r="G111" s="107"/>
-      <c r="H111" s="107"/>
-      <c r="I111" s="107"/>
-      <c r="J111" s="107"/>
-      <c r="K111" s="107"/>
+      <c r="G111" s="107">
+        <f>(-G109-G110+G112)/-1</f>
+        <v>-647.56000000000131</v>
+      </c>
+      <c r="H111" s="107">
+        <f t="shared" ref="H111:K111" si="56">(-H109-H110+H112)/-1</f>
+        <v>-2914.7136000000028</v>
+      </c>
+      <c r="I111" s="107">
+        <f t="shared" si="56"/>
+        <v>-3308.3539583999991</v>
+      </c>
+      <c r="J111" s="107">
+        <f t="shared" si="56"/>
+        <v>-3536.6303815296014</v>
+      </c>
+      <c r="K111" s="107">
+        <f t="shared" si="56"/>
+        <v>-3780.6578778551411</v>
+      </c>
       <c r="M111" t="s">
         <v>167</v>
       </c>
@@ -55263,32 +55633,32 @@
         <v>28</v>
       </c>
       <c r="E112" s="29">
-        <f t="shared" ref="E112:K112" si="33">E50</f>
+        <f t="shared" ref="E112:K112" si="57">E50</f>
         <v>18177</v>
       </c>
       <c r="F112" s="29">
-        <f t="shared" si="33"/>
+        <f t="shared" si="57"/>
         <v>22283</v>
       </c>
       <c r="G112" s="29">
-        <f t="shared" si="33"/>
-        <v>22283.96</v>
+        <f t="shared" si="57"/>
+        <v>21391.68</v>
       </c>
       <c r="H112" s="29">
-        <f t="shared" si="33"/>
-        <v>22285.02</v>
+        <f t="shared" si="57"/>
+        <v>22675.180800000002</v>
       </c>
       <c r="I112" s="29">
-        <f t="shared" si="33"/>
-        <v>22286.089</v>
+        <f t="shared" si="57"/>
+        <v>24239.7682752</v>
       </c>
       <c r="J112" s="29">
-        <f t="shared" si="33"/>
-        <v>22287.157999999999</v>
+        <f t="shared" si="57"/>
+        <v>25912.3122861888</v>
       </c>
       <c r="K112" s="29">
-        <f t="shared" si="33"/>
-        <v>22288.226999999999</v>
+        <f t="shared" si="57"/>
+        <v>27700.261833935827</v>
       </c>
       <c r="M112" t="s">
         <v>168</v>

</xml_diff>